<commit_message>
quantity now calculated base on weekly prodcution
</commit_message>
<xml_diff>
--- a/Viajante/BD/FLUXO.xlsx
+++ b/Viajante/BD/FLUXO.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\perna\Desktop\STALLANTIS\VIAJANTE - ENGENHARIA\Viajante-Engenharia\BD\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\perna\Desktop\STALLANTIS\BC TURBO\BC Turbo App\Viajante\BD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75784411-EF89-440D-9F94-AF61E7098FC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A15F0B56-5FB7-4870-86D8-AB785A964374}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-2445" windowWidth="21840" windowHeight="13020" xr2:uid="{560AD881-1239-4AD1-960A-2C71473C6A4C}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{560AD881-1239-4AD1-960A-2C71473C6A4C}"/>
   </bookViews>
   <sheets>
     <sheet name="FLUXOS" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2315" uniqueCount="193">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2323" uniqueCount="195">
   <si>
     <t>COD FLUXO</t>
   </si>
@@ -621,6 +621,12 @@
   </si>
   <si>
     <t>800005740, 800035411</t>
+  </si>
+  <si>
+    <t>DANA II</t>
+  </si>
+  <si>
+    <t>TRUCK SIDER</t>
   </si>
 </sst>
 </file>
@@ -974,7 +980,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B90B9044-5A84-4453-A4AB-9D3FAB58BBA5}">
-  <dimension ref="A1:L140"/>
+  <dimension ref="A1:L141"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="7.6328125" style="2" bestFit="1" customWidth="1"/>
@@ -6283,7 +6289,46 @@
         <v>96</v>
       </c>
     </row>
+    <row r="141" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A141" s="2">
+        <v>192</v>
+      </c>
+      <c r="B141" s="2">
+        <v>11568</v>
+      </c>
+      <c r="C141" s="2">
+        <v>800002588</v>
+      </c>
+      <c r="D141" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="E141" s="2">
+        <v>1128</v>
+      </c>
+      <c r="F141" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="G141" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="H141" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I141" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="J141" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="K141" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="L141" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
   </sheetData>
+  <autoFilter ref="A1:L140" xr:uid="{B90B9044-5A84-4453-A4AB-9D3FAB58BBA5}"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
 </file>
@@ -11685,6 +11730,7 @@
 
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{725ca717-11da-4935-b601-f527b9741f2e}" enabled="1" method="Standard" siteId="{d852d5cd-724c-4128-8812-ffa5db3f8507}" contentBits="0" removed="0"/>
   <clbl:label id="{736915f3-2f02-4945-8997-f2963298db46}" enabled="1" method="Standard" siteId="{cd99fef8-1cd3-4a2a-9bdf-15531181d65e}" contentBits="1" removed="0"/>
 </clbl:labelList>
 </file>
</xml_diff>

<commit_message>
The AS IS qtde has been updated and working corectly, need some simple validations and tests
</commit_message>
<xml_diff>
--- a/Viajante/BD/FLUXO.xlsx
+++ b/Viajante/BD/FLUXO.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\perna\Desktop\STALLANTIS\BC TURBO\BC Turbo App\Viajante\BD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A15F0B56-5FB7-4870-86D8-AB785A964374}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCD65E6C-1851-4E71-BF62-BBE5752BF57E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{560AD881-1239-4AD1-960A-2C71473C6A4C}"/>
+    <workbookView minimized="1" xWindow="5230" yWindow="3230" windowWidth="14400" windowHeight="7280" xr2:uid="{560AD881-1239-4AD1-960A-2C71473C6A4C}"/>
   </bookViews>
   <sheets>
     <sheet name="FLUXOS" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Base Forncedores'!$A$1:$L$140</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">FLUXOS!$A$1:$L$140</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">FLUXOS!$A$1:$L$141</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2323" uniqueCount="195">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2323" uniqueCount="196">
   <si>
     <t>COD FLUXO</t>
   </si>
@@ -627,6 +627,9 @@
   </si>
   <si>
     <t>TRUCK SIDER</t>
+  </si>
+  <si>
+    <t>CARRETA SIDER</t>
   </si>
 </sst>
 </file>
@@ -980,6 +983,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B90B9044-5A84-4453-A4AB-9D3FAB58BBA5}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:L141"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -1035,7 +1039,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -1073,7 +1077,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="3" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -1111,7 +1115,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -1149,7 +1153,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -1187,7 +1191,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -1225,7 +1229,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -1263,7 +1267,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="8" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -1301,7 +1305,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A9" s="2">
         <v>8</v>
       </c>
@@ -1339,7 +1343,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="10" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A10" s="2">
         <v>9</v>
       </c>
@@ -1377,7 +1381,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A11" s="2">
         <v>20</v>
       </c>
@@ -1415,7 +1419,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="12" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A12" s="2">
         <v>21</v>
       </c>
@@ -1473,7 +1477,7 @@
         <v>27</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>50</v>
+        <v>195</v>
       </c>
       <c r="H13" s="2" t="s">
         <v>12</v>
@@ -1491,7 +1495,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="14" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A14" s="2">
         <v>23</v>
       </c>
@@ -1529,7 +1533,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="15" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A15" s="2">
         <v>24</v>
       </c>
@@ -1567,7 +1571,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="16" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A16" s="2">
         <v>25</v>
       </c>
@@ -1605,7 +1609,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="17" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A17" s="2">
         <v>26</v>
       </c>
@@ -1643,7 +1647,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="18" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A18" s="2">
         <v>27</v>
       </c>
@@ -1681,7 +1685,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="19" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A19" s="2">
         <v>28</v>
       </c>
@@ -1719,7 +1723,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="20" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A20" s="2">
         <v>31</v>
       </c>
@@ -1757,7 +1761,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="21" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A21" s="2">
         <v>33</v>
       </c>
@@ -1795,7 +1799,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="22" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A22" s="2">
         <v>34</v>
       </c>
@@ -1833,7 +1837,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="23" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A23" s="2">
         <v>35</v>
       </c>
@@ -1871,7 +1875,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="24" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A24" s="2">
         <v>37</v>
       </c>
@@ -1909,7 +1913,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="25" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A25" s="2">
         <v>38</v>
       </c>
@@ -1947,7 +1951,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="26" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A26" s="2">
         <v>39</v>
       </c>
@@ -1985,7 +1989,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="27" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A27" s="2">
         <v>40</v>
       </c>
@@ -2023,7 +2027,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="28" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A28" s="2">
         <v>41</v>
       </c>
@@ -2061,7 +2065,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="29" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A29" s="2">
         <v>42</v>
       </c>
@@ -2099,7 +2103,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="30" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A30" s="2">
         <v>43</v>
       </c>
@@ -2137,7 +2141,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="31" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A31" s="2">
         <v>44</v>
       </c>
@@ -2175,7 +2179,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="32" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A32" s="2">
         <v>48</v>
       </c>
@@ -2213,7 +2217,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="33" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A33" s="2">
         <v>49</v>
       </c>
@@ -2251,7 +2255,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="34" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A34" s="2">
         <v>50</v>
       </c>
@@ -2289,7 +2293,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="35" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A35" s="2">
         <v>51</v>
       </c>
@@ -2327,7 +2331,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="36" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A36" s="2">
         <v>52</v>
       </c>
@@ -2365,7 +2369,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="37" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A37" s="2">
         <v>54</v>
       </c>
@@ -2403,7 +2407,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="38" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A38" s="2">
         <v>55</v>
       </c>
@@ -2441,7 +2445,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="39" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A39" s="2">
         <v>57</v>
       </c>
@@ -2479,7 +2483,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="40" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A40" s="2">
         <v>58</v>
       </c>
@@ -2517,7 +2521,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="41" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A41" s="2">
         <v>60</v>
       </c>
@@ -2555,7 +2559,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="42" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A42" s="2">
         <v>61</v>
       </c>
@@ -2593,7 +2597,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="43" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A43" s="2">
         <v>62</v>
       </c>
@@ -2631,7 +2635,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="44" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A44" s="2">
         <v>63</v>
       </c>
@@ -2669,7 +2673,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="45" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A45" s="2">
         <v>64</v>
       </c>
@@ -2707,7 +2711,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="46" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A46" s="2">
         <v>66</v>
       </c>
@@ -2745,7 +2749,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="47" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A47" s="2">
         <v>67</v>
       </c>
@@ -2783,7 +2787,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="48" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A48" s="2">
         <v>68</v>
       </c>
@@ -2821,7 +2825,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="49" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A49" s="2">
         <v>70</v>
       </c>
@@ -2859,7 +2863,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="50" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A50" s="2">
         <v>71</v>
       </c>
@@ -2897,7 +2901,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="51" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A51" s="2">
         <v>74</v>
       </c>
@@ -2935,7 +2939,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="52" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A52" s="2">
         <v>75</v>
       </c>
@@ -2973,7 +2977,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="53" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A53" s="2">
         <v>76</v>
       </c>
@@ -3011,7 +3015,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="54" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A54" s="2">
         <v>77</v>
       </c>
@@ -3049,7 +3053,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="55" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A55" s="2">
         <v>79</v>
       </c>
@@ -3087,7 +3091,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="56" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A56" s="2">
         <v>81</v>
       </c>
@@ -3125,7 +3129,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="57" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A57" s="2">
         <v>82</v>
       </c>
@@ -3163,7 +3167,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="58" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A58" s="2">
         <v>83</v>
       </c>
@@ -3201,7 +3205,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="59" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A59" s="2">
         <v>85</v>
       </c>
@@ -3239,7 +3243,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="60" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A60" s="2">
         <v>86</v>
       </c>
@@ -3277,7 +3281,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="61" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A61" s="2">
         <v>87</v>
       </c>
@@ -3315,7 +3319,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="62" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A62" s="2">
         <v>88</v>
       </c>
@@ -3353,7 +3357,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="63" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A63" s="2">
         <v>89</v>
       </c>
@@ -3391,7 +3395,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="64" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A64" s="2">
         <v>90</v>
       </c>
@@ -3429,7 +3433,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="65" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A65" s="2">
         <v>91</v>
       </c>
@@ -3467,7 +3471,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="66" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A66" s="2">
         <v>92</v>
       </c>
@@ -3505,7 +3509,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="67" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A67" s="2">
         <v>93</v>
       </c>
@@ -3543,7 +3547,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="68" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A68" s="2">
         <v>94</v>
       </c>
@@ -3581,7 +3585,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="69" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A69" s="2">
         <v>95</v>
       </c>
@@ -3619,7 +3623,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="70" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A70" s="2">
         <v>96</v>
       </c>
@@ -3657,7 +3661,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="71" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A71" s="2">
         <v>100</v>
       </c>
@@ -3695,7 +3699,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="72" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A72" s="2">
         <v>101</v>
       </c>
@@ -3733,7 +3737,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="73" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A73" s="2">
         <v>102</v>
       </c>
@@ -3771,7 +3775,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="74" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A74" s="2">
         <v>105</v>
       </c>
@@ -3809,7 +3813,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="75" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A75" s="2">
         <v>107</v>
       </c>
@@ -3847,7 +3851,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="76" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A76" s="2">
         <v>108</v>
       </c>
@@ -3885,7 +3889,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="77" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A77" s="2">
         <v>110</v>
       </c>
@@ -3923,7 +3927,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="78" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A78" s="2">
         <v>112</v>
       </c>
@@ -3961,7 +3965,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="79" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A79" s="2">
         <v>113</v>
       </c>
@@ -3999,7 +4003,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="80" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A80" s="2">
         <v>114</v>
       </c>
@@ -4037,7 +4041,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="81" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A81" s="2">
         <v>116</v>
       </c>
@@ -4075,7 +4079,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="82" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A82" s="2">
         <v>119</v>
       </c>
@@ -4113,7 +4117,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="83" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A83" s="2">
         <v>120</v>
       </c>
@@ -4151,7 +4155,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="84" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A84" s="2">
         <v>122</v>
       </c>
@@ -4189,7 +4193,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="85" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A85" s="2">
         <v>123</v>
       </c>
@@ -4227,7 +4231,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="86" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A86" s="2">
         <v>169</v>
       </c>
@@ -4265,7 +4269,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="87" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A87" s="2">
         <v>124</v>
       </c>
@@ -4303,7 +4307,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="88" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A88" s="2">
         <v>125</v>
       </c>
@@ -4341,7 +4345,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="89" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A89" s="2">
         <v>126</v>
       </c>
@@ -4379,7 +4383,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="90" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A90" s="2">
         <v>127</v>
       </c>
@@ -4417,7 +4421,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="91" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A91" s="2">
         <v>128</v>
       </c>
@@ -4455,7 +4459,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="92" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A92" s="2">
         <v>129</v>
       </c>
@@ -4493,7 +4497,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="93" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A93" s="2">
         <v>130</v>
       </c>
@@ -4531,7 +4535,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="94" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A94" s="2">
         <v>132</v>
       </c>
@@ -4569,7 +4573,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="95" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A95" s="2">
         <v>133</v>
       </c>
@@ -4607,7 +4611,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="96" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A96" s="2">
         <v>134</v>
       </c>
@@ -4645,7 +4649,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="97" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A97" s="2">
         <v>136</v>
       </c>
@@ -4683,7 +4687,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="98" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A98" s="2">
         <v>138</v>
       </c>
@@ -4721,7 +4725,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="99" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A99" s="2">
         <v>140</v>
       </c>
@@ -4759,7 +4763,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="100" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A100" s="2">
         <v>141</v>
       </c>
@@ -4797,7 +4801,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="101" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A101" s="2">
         <v>142</v>
       </c>
@@ -4835,7 +4839,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="102" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A102" s="2">
         <v>143</v>
       </c>
@@ -4873,7 +4877,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="103" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A103" s="2">
         <v>144</v>
       </c>
@@ -4911,7 +4915,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="104" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A104" s="2">
         <v>145</v>
       </c>
@@ -4949,7 +4953,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="105" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A105" s="2">
         <v>148</v>
       </c>
@@ -4987,7 +4991,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="106" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A106" s="2">
         <v>156</v>
       </c>
@@ -5023,7 +5027,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="107" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A107" s="2">
         <v>157</v>
       </c>
@@ -5059,7 +5063,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="108" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A108" s="2">
         <v>158</v>
       </c>
@@ -5097,7 +5101,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="109" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A109" s="2">
         <v>159</v>
       </c>
@@ -5133,7 +5137,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="110" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A110" s="2">
         <v>160</v>
       </c>
@@ -5169,7 +5173,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="111" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A111" s="2">
         <v>161</v>
       </c>
@@ -5205,7 +5209,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="112" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A112" s="2">
         <v>162</v>
       </c>
@@ -5241,7 +5245,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="113" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A113" s="2">
         <v>163</v>
       </c>
@@ -5277,7 +5281,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="114" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A114" s="2">
         <v>164</v>
       </c>
@@ -5313,7 +5317,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="115" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A115" s="2">
         <v>165</v>
       </c>
@@ -5351,7 +5355,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="116" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A116" s="2">
         <v>166</v>
       </c>
@@ -5387,7 +5391,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="117" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A117" s="2">
         <v>167</v>
       </c>
@@ -5423,7 +5427,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="118" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A118" s="2">
         <v>168</v>
       </c>
@@ -5461,7 +5465,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="119" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A119" s="2">
         <v>170</v>
       </c>
@@ -5499,7 +5503,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="120" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A120" s="2">
         <v>171</v>
       </c>
@@ -5537,7 +5541,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="121" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A121" s="2">
         <v>172</v>
       </c>
@@ -5575,7 +5579,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="122" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A122" s="2">
         <v>173</v>
       </c>
@@ -5613,7 +5617,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="123" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A123" s="2">
         <v>174</v>
       </c>
@@ -5651,7 +5655,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="124" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A124" s="2">
         <v>175</v>
       </c>
@@ -5689,7 +5693,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="125" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A125" s="2">
         <v>176</v>
       </c>
@@ -5727,7 +5731,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="126" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A126" s="2">
         <v>177</v>
       </c>
@@ -5765,7 +5769,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="127" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A127" s="2">
         <v>178</v>
       </c>
@@ -5803,7 +5807,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="128" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A128" s="2">
         <v>179</v>
       </c>
@@ -5841,7 +5845,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="129" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A129" s="2">
         <v>180</v>
       </c>
@@ -5879,7 +5883,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="130" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A130" s="2">
         <v>181</v>
       </c>
@@ -5917,7 +5921,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="131" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A131" s="2">
         <v>182</v>
       </c>
@@ -5955,7 +5959,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="132" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A132" s="2">
         <v>183</v>
       </c>
@@ -5993,7 +5997,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="133" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A133" s="2">
         <v>184</v>
       </c>
@@ -6029,7 +6033,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="134" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A134" s="2">
         <v>185</v>
       </c>
@@ -6065,7 +6069,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="135" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A135" s="2">
         <v>186</v>
       </c>
@@ -6101,7 +6105,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="136" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A136" s="2">
         <v>187</v>
       </c>
@@ -6137,7 +6141,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="137" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A137" s="2">
         <v>188</v>
       </c>
@@ -6175,7 +6179,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="138" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A138" s="2">
         <v>189</v>
       </c>
@@ -6213,7 +6217,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="139" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A139" s="2">
         <v>190</v>
       </c>
@@ -6251,7 +6255,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="140" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A140" s="2">
         <v>191</v>
       </c>
@@ -6289,7 +6293,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="141" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A141" s="2">
         <v>192</v>
       </c>
@@ -6328,7 +6332,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L140" xr:uid="{B90B9044-5A84-4453-A4AB-9D3FAB58BBA5}"/>
+  <autoFilter ref="A1:L141" xr:uid="{B90B9044-5A84-4453-A4AB-9D3FAB58BBA5}">
+    <filterColumn colId="3">
+      <filters>
+        <filter val="COOPER STANDARD"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
checking why COD IMS and SAP not use for the template
</commit_message>
<xml_diff>
--- a/Viajante/BD/FLUXO.xlsx
+++ b/Viajante/BD/FLUXO.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\perna\Desktop\STALLANTIS\BC TURBO\BC Turbo App\Viajante\BD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCD65E6C-1851-4E71-BF62-BBE5752BF57E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A35D2919-3134-4C65-86E7-7E53F04C3F5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="5230" yWindow="3230" windowWidth="14400" windowHeight="7280" xr2:uid="{560AD881-1239-4AD1-960A-2C71473C6A4C}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{560AD881-1239-4AD1-960A-2C71473C6A4C}"/>
   </bookViews>
   <sheets>
     <sheet name="FLUXOS" sheetId="1" r:id="rId1"/>
@@ -983,7 +983,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B90B9044-5A84-4453-A4AB-9D3FAB58BBA5}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:L141"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -1039,7 +1038,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -1077,7 +1076,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="3" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -1115,7 +1114,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -1153,7 +1152,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -1191,7 +1190,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -1229,7 +1228,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -1267,7 +1266,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="8" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -1305,7 +1304,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A9" s="2">
         <v>8</v>
       </c>
@@ -1343,7 +1342,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="10" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A10" s="2">
         <v>9</v>
       </c>
@@ -1381,7 +1380,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A11" s="2">
         <v>20</v>
       </c>
@@ -1419,7 +1418,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="12" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A12" s="2">
         <v>21</v>
       </c>
@@ -1495,7 +1494,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="14" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A14" s="2">
         <v>23</v>
       </c>
@@ -1533,7 +1532,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="15" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A15" s="2">
         <v>24</v>
       </c>
@@ -1571,7 +1570,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="16" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A16" s="2">
         <v>25</v>
       </c>
@@ -1609,7 +1608,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="17" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A17" s="2">
         <v>26</v>
       </c>
@@ -1647,7 +1646,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="18" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A18" s="2">
         <v>27</v>
       </c>
@@ -1685,7 +1684,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="19" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A19" s="2">
         <v>28</v>
       </c>
@@ -1723,7 +1722,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="20" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A20" s="2">
         <v>31</v>
       </c>
@@ -1761,7 +1760,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="21" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A21" s="2">
         <v>33</v>
       </c>
@@ -1799,7 +1798,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="22" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A22" s="2">
         <v>34</v>
       </c>
@@ -1837,7 +1836,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="23" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A23" s="2">
         <v>35</v>
       </c>
@@ -1875,7 +1874,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="24" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A24" s="2">
         <v>37</v>
       </c>
@@ -1913,7 +1912,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="25" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A25" s="2">
         <v>38</v>
       </c>
@@ -1951,7 +1950,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="26" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A26" s="2">
         <v>39</v>
       </c>
@@ -1989,7 +1988,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="27" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A27" s="2">
         <v>40</v>
       </c>
@@ -2027,7 +2026,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="28" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A28" s="2">
         <v>41</v>
       </c>
@@ -2065,7 +2064,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="29" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A29" s="2">
         <v>42</v>
       </c>
@@ -2103,7 +2102,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="30" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A30" s="2">
         <v>43</v>
       </c>
@@ -2141,7 +2140,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="31" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A31" s="2">
         <v>44</v>
       </c>
@@ -2179,7 +2178,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="32" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A32" s="2">
         <v>48</v>
       </c>
@@ -2217,7 +2216,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="33" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A33" s="2">
         <v>49</v>
       </c>
@@ -2255,7 +2254,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="34" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A34" s="2">
         <v>50</v>
       </c>
@@ -2293,7 +2292,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="35" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A35" s="2">
         <v>51</v>
       </c>
@@ -2331,7 +2330,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="36" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A36" s="2">
         <v>52</v>
       </c>
@@ -2369,7 +2368,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="37" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A37" s="2">
         <v>54</v>
       </c>
@@ -2407,7 +2406,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="38" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A38" s="2">
         <v>55</v>
       </c>
@@ -2445,7 +2444,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="39" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A39" s="2">
         <v>57</v>
       </c>
@@ -2483,7 +2482,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="40" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A40" s="2">
         <v>58</v>
       </c>
@@ -2521,7 +2520,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="41" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A41" s="2">
         <v>60</v>
       </c>
@@ -2559,7 +2558,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="42" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A42" s="2">
         <v>61</v>
       </c>
@@ -2597,7 +2596,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="43" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A43" s="2">
         <v>62</v>
       </c>
@@ -2635,7 +2634,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="44" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A44" s="2">
         <v>63</v>
       </c>
@@ -2673,7 +2672,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="45" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A45" s="2">
         <v>64</v>
       </c>
@@ -2711,7 +2710,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="46" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A46" s="2">
         <v>66</v>
       </c>
@@ -2749,7 +2748,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="47" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A47" s="2">
         <v>67</v>
       </c>
@@ -2787,7 +2786,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="48" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A48" s="2">
         <v>68</v>
       </c>
@@ -2825,7 +2824,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="49" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A49" s="2">
         <v>70</v>
       </c>
@@ -2863,7 +2862,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="50" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A50" s="2">
         <v>71</v>
       </c>
@@ -2901,7 +2900,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="51" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A51" s="2">
         <v>74</v>
       </c>
@@ -2939,7 +2938,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="52" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A52" s="2">
         <v>75</v>
       </c>
@@ -2977,7 +2976,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="53" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A53" s="2">
         <v>76</v>
       </c>
@@ -3015,7 +3014,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="54" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A54" s="2">
         <v>77</v>
       </c>
@@ -3053,7 +3052,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="55" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A55" s="2">
         <v>79</v>
       </c>
@@ -3091,7 +3090,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="56" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A56" s="2">
         <v>81</v>
       </c>
@@ -3129,7 +3128,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="57" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A57" s="2">
         <v>82</v>
       </c>
@@ -3167,7 +3166,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="58" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A58" s="2">
         <v>83</v>
       </c>
@@ -3205,7 +3204,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="59" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A59" s="2">
         <v>85</v>
       </c>
@@ -3243,7 +3242,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="60" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A60" s="2">
         <v>86</v>
       </c>
@@ -3281,7 +3280,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="61" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A61" s="2">
         <v>87</v>
       </c>
@@ -3319,7 +3318,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="62" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A62" s="2">
         <v>88</v>
       </c>
@@ -3357,7 +3356,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="63" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A63" s="2">
         <v>89</v>
       </c>
@@ -3395,7 +3394,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="64" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A64" s="2">
         <v>90</v>
       </c>
@@ -3433,7 +3432,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="65" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A65" s="2">
         <v>91</v>
       </c>
@@ -3471,7 +3470,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="66" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A66" s="2">
         <v>92</v>
       </c>
@@ -3509,7 +3508,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="67" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A67" s="2">
         <v>93</v>
       </c>
@@ -3547,7 +3546,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="68" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A68" s="2">
         <v>94</v>
       </c>
@@ -3585,7 +3584,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="69" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A69" s="2">
         <v>95</v>
       </c>
@@ -3623,7 +3622,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="70" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A70" s="2">
         <v>96</v>
       </c>
@@ -3661,7 +3660,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="71" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A71" s="2">
         <v>100</v>
       </c>
@@ -3699,7 +3698,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="72" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A72" s="2">
         <v>101</v>
       </c>
@@ -3737,7 +3736,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="73" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A73" s="2">
         <v>102</v>
       </c>
@@ -3775,7 +3774,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="74" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A74" s="2">
         <v>105</v>
       </c>
@@ -3813,7 +3812,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="75" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A75" s="2">
         <v>107</v>
       </c>
@@ -3851,7 +3850,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="76" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A76" s="2">
         <v>108</v>
       </c>
@@ -3889,7 +3888,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="77" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A77" s="2">
         <v>110</v>
       </c>
@@ -3927,7 +3926,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="78" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A78" s="2">
         <v>112</v>
       </c>
@@ -3965,7 +3964,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="79" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A79" s="2">
         <v>113</v>
       </c>
@@ -4003,7 +4002,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="80" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A80" s="2">
         <v>114</v>
       </c>
@@ -4041,7 +4040,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="81" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A81" s="2">
         <v>116</v>
       </c>
@@ -4079,7 +4078,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="82" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A82" s="2">
         <v>119</v>
       </c>
@@ -4117,7 +4116,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="83" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A83" s="2">
         <v>120</v>
       </c>
@@ -4155,7 +4154,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="84" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A84" s="2">
         <v>122</v>
       </c>
@@ -4193,7 +4192,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="85" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A85" s="2">
         <v>123</v>
       </c>
@@ -4231,7 +4230,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="86" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A86" s="2">
         <v>169</v>
       </c>
@@ -4269,7 +4268,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="87" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A87" s="2">
         <v>124</v>
       </c>
@@ -4307,7 +4306,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="88" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A88" s="2">
         <v>125</v>
       </c>
@@ -4345,7 +4344,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="89" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A89" s="2">
         <v>126</v>
       </c>
@@ -4383,7 +4382,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="90" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A90" s="2">
         <v>127</v>
       </c>
@@ -4421,7 +4420,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="91" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A91" s="2">
         <v>128</v>
       </c>
@@ -4459,7 +4458,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="92" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A92" s="2">
         <v>129</v>
       </c>
@@ -4497,7 +4496,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="93" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A93" s="2">
         <v>130</v>
       </c>
@@ -4535,7 +4534,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="94" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A94" s="2">
         <v>132</v>
       </c>
@@ -4573,7 +4572,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="95" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A95" s="2">
         <v>133</v>
       </c>
@@ -4611,7 +4610,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="96" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A96" s="2">
         <v>134</v>
       </c>
@@ -4649,7 +4648,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="97" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A97" s="2">
         <v>136</v>
       </c>
@@ -4687,7 +4686,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="98" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A98" s="2">
         <v>138</v>
       </c>
@@ -4725,7 +4724,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="99" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A99" s="2">
         <v>140</v>
       </c>
@@ -4763,7 +4762,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="100" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A100" s="2">
         <v>141</v>
       </c>
@@ -4801,7 +4800,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="101" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A101" s="2">
         <v>142</v>
       </c>
@@ -4839,7 +4838,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="102" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A102" s="2">
         <v>143</v>
       </c>
@@ -4877,7 +4876,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="103" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A103" s="2">
         <v>144</v>
       </c>
@@ -4915,7 +4914,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="104" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A104" s="2">
         <v>145</v>
       </c>
@@ -4953,7 +4952,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="105" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A105" s="2">
         <v>148</v>
       </c>
@@ -4991,7 +4990,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="106" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A106" s="2">
         <v>156</v>
       </c>
@@ -5027,7 +5026,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="107" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A107" s="2">
         <v>157</v>
       </c>
@@ -5063,7 +5062,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="108" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A108" s="2">
         <v>158</v>
       </c>
@@ -5101,7 +5100,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="109" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A109" s="2">
         <v>159</v>
       </c>
@@ -5137,7 +5136,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="110" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A110" s="2">
         <v>160</v>
       </c>
@@ -5173,7 +5172,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="111" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A111" s="2">
         <v>161</v>
       </c>
@@ -5209,7 +5208,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="112" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A112" s="2">
         <v>162</v>
       </c>
@@ -5245,7 +5244,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="113" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A113" s="2">
         <v>163</v>
       </c>
@@ -5281,7 +5280,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="114" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A114" s="2">
         <v>164</v>
       </c>
@@ -5317,7 +5316,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="115" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A115" s="2">
         <v>165</v>
       </c>
@@ -5355,7 +5354,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="116" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A116" s="2">
         <v>166</v>
       </c>
@@ -5391,7 +5390,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="117" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A117" s="2">
         <v>167</v>
       </c>
@@ -5427,7 +5426,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="118" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A118" s="2">
         <v>168</v>
       </c>
@@ -5465,7 +5464,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="119" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A119" s="2">
         <v>170</v>
       </c>
@@ -5503,7 +5502,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="120" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A120" s="2">
         <v>171</v>
       </c>
@@ -5541,7 +5540,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="121" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A121" s="2">
         <v>172</v>
       </c>
@@ -5579,7 +5578,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="122" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A122" s="2">
         <v>173</v>
       </c>
@@ -5617,7 +5616,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="123" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A123" s="2">
         <v>174</v>
       </c>
@@ -5655,7 +5654,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="124" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A124" s="2">
         <v>175</v>
       </c>
@@ -5693,7 +5692,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="125" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A125" s="2">
         <v>176</v>
       </c>
@@ -5731,7 +5730,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="126" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A126" s="2">
         <v>177</v>
       </c>
@@ -5769,7 +5768,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="127" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A127" s="2">
         <v>178</v>
       </c>
@@ -5807,7 +5806,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="128" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A128" s="2">
         <v>179</v>
       </c>
@@ -5845,7 +5844,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="129" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A129" s="2">
         <v>180</v>
       </c>
@@ -5883,7 +5882,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="130" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A130" s="2">
         <v>181</v>
       </c>
@@ -5921,7 +5920,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="131" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A131" s="2">
         <v>182</v>
       </c>
@@ -5959,7 +5958,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="132" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A132" s="2">
         <v>183</v>
       </c>
@@ -5997,7 +5996,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="133" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A133" s="2">
         <v>184</v>
       </c>
@@ -6033,7 +6032,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="134" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A134" s="2">
         <v>185</v>
       </c>
@@ -6069,7 +6068,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="135" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A135" s="2">
         <v>186</v>
       </c>
@@ -6105,7 +6104,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="136" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A136" s="2">
         <v>187</v>
       </c>
@@ -6141,7 +6140,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="137" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A137" s="2">
         <v>188</v>
       </c>
@@ -6179,7 +6178,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="138" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A138" s="2">
         <v>189</v>
       </c>
@@ -6217,7 +6216,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="139" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A139" s="2">
         <v>190</v>
       </c>
@@ -6255,7 +6254,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="140" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A140" s="2">
         <v>191</v>
       </c>
@@ -6293,7 +6292,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="141" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A141" s="2">
         <v>192</v>
       </c>
@@ -6332,13 +6331,6 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L141" xr:uid="{B90B9044-5A84-4453-A4AB-9D3FAB58BBA5}">
-    <filterColumn colId="3">
-      <filters>
-        <filter val="COOPER STANDARD"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Custo is OK and need to check how pedagio will be calculated and verufy the other options
</commit_message>
<xml_diff>
--- a/Viajante/BD/FLUXO.xlsx
+++ b/Viajante/BD/FLUXO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\perna\Desktop\STALLANTIS\BC TURBO\BC Turbo App\Viajante\BD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A35D2919-3134-4C65-86E7-7E53F04C3F5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88C0621D-F0FB-4B71-BF54-5C7DAA410E63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{560AD881-1239-4AD1-960A-2C71473C6A4C}"/>
   </bookViews>
@@ -983,6 +983,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B90B9044-5A84-4453-A4AB-9D3FAB58BBA5}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:L141"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -1038,7 +1039,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -1076,7 +1077,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="3" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -1114,7 +1115,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -1152,7 +1153,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -1190,7 +1191,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -1228,7 +1229,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -1266,7 +1267,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="8" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -1304,7 +1305,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A9" s="2">
         <v>8</v>
       </c>
@@ -1342,7 +1343,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="10" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A10" s="2">
         <v>9</v>
       </c>
@@ -1380,7 +1381,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A11" s="2">
         <v>20</v>
       </c>
@@ -1418,7 +1419,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="12" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A12" s="2">
         <v>21</v>
       </c>
@@ -1494,7 +1495,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="14" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A14" s="2">
         <v>23</v>
       </c>
@@ -1532,7 +1533,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="15" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A15" s="2">
         <v>24</v>
       </c>
@@ -1570,7 +1571,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="16" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A16" s="2">
         <v>25</v>
       </c>
@@ -1608,7 +1609,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="17" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A17" s="2">
         <v>26</v>
       </c>
@@ -1646,7 +1647,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="18" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A18" s="2">
         <v>27</v>
       </c>
@@ -1684,7 +1685,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="19" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A19" s="2">
         <v>28</v>
       </c>
@@ -1722,7 +1723,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="20" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A20" s="2">
         <v>31</v>
       </c>
@@ -1760,7 +1761,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="21" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A21" s="2">
         <v>33</v>
       </c>
@@ -1798,7 +1799,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="22" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A22" s="2">
         <v>34</v>
       </c>
@@ -1836,7 +1837,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="23" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A23" s="2">
         <v>35</v>
       </c>
@@ -1874,7 +1875,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="24" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A24" s="2">
         <v>37</v>
       </c>
@@ -1912,7 +1913,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="25" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A25" s="2">
         <v>38</v>
       </c>
@@ -1950,7 +1951,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="26" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A26" s="2">
         <v>39</v>
       </c>
@@ -1988,7 +1989,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="27" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A27" s="2">
         <v>40</v>
       </c>
@@ -2026,7 +2027,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="28" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A28" s="2">
         <v>41</v>
       </c>
@@ -2064,7 +2065,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="29" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A29" s="2">
         <v>42</v>
       </c>
@@ -2102,7 +2103,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="30" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A30" s="2">
         <v>43</v>
       </c>
@@ -2140,7 +2141,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="31" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A31" s="2">
         <v>44</v>
       </c>
@@ -2178,7 +2179,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="32" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A32" s="2">
         <v>48</v>
       </c>
@@ -2216,7 +2217,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="33" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A33" s="2">
         <v>49</v>
       </c>
@@ -2254,7 +2255,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="34" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A34" s="2">
         <v>50</v>
       </c>
@@ -2292,7 +2293,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="35" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A35" s="2">
         <v>51</v>
       </c>
@@ -2330,7 +2331,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="36" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A36" s="2">
         <v>52</v>
       </c>
@@ -2368,7 +2369,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="37" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A37" s="2">
         <v>54</v>
       </c>
@@ -2406,7 +2407,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="38" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A38" s="2">
         <v>55</v>
       </c>
@@ -2444,7 +2445,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="39" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A39" s="2">
         <v>57</v>
       </c>
@@ -2482,7 +2483,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="40" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A40" s="2">
         <v>58</v>
       </c>
@@ -2520,7 +2521,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="41" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A41" s="2">
         <v>60</v>
       </c>
@@ -2558,7 +2559,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="42" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A42" s="2">
         <v>61</v>
       </c>
@@ -2596,7 +2597,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="43" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A43" s="2">
         <v>62</v>
       </c>
@@ -2634,7 +2635,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="44" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A44" s="2">
         <v>63</v>
       </c>
@@ -2672,7 +2673,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="45" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A45" s="2">
         <v>64</v>
       </c>
@@ -2710,7 +2711,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="46" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A46" s="2">
         <v>66</v>
       </c>
@@ -2748,7 +2749,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="47" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A47" s="2">
         <v>67</v>
       </c>
@@ -2786,7 +2787,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="48" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A48" s="2">
         <v>68</v>
       </c>
@@ -2824,7 +2825,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="49" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A49" s="2">
         <v>70</v>
       </c>
@@ -2862,7 +2863,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="50" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A50" s="2">
         <v>71</v>
       </c>
@@ -2900,7 +2901,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="51" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A51" s="2">
         <v>74</v>
       </c>
@@ -2938,7 +2939,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="52" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A52" s="2">
         <v>75</v>
       </c>
@@ -2976,7 +2977,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="53" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A53" s="2">
         <v>76</v>
       </c>
@@ -3014,7 +3015,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="54" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A54" s="2">
         <v>77</v>
       </c>
@@ -3052,7 +3053,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="55" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A55" s="2">
         <v>79</v>
       </c>
@@ -3090,7 +3091,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="56" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A56" s="2">
         <v>81</v>
       </c>
@@ -3128,7 +3129,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="57" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A57" s="2">
         <v>82</v>
       </c>
@@ -3166,7 +3167,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="58" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A58" s="2">
         <v>83</v>
       </c>
@@ -3204,7 +3205,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="59" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A59" s="2">
         <v>85</v>
       </c>
@@ -3242,7 +3243,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="60" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A60" s="2">
         <v>86</v>
       </c>
@@ -3280,7 +3281,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="61" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A61" s="2">
         <v>87</v>
       </c>
@@ -3318,7 +3319,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="62" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A62" s="2">
         <v>88</v>
       </c>
@@ -3356,7 +3357,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="63" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A63" s="2">
         <v>89</v>
       </c>
@@ -3394,7 +3395,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="64" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A64" s="2">
         <v>90</v>
       </c>
@@ -3432,7 +3433,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="65" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A65" s="2">
         <v>91</v>
       </c>
@@ -3470,7 +3471,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="66" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A66" s="2">
         <v>92</v>
       </c>
@@ -3508,7 +3509,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="67" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A67" s="2">
         <v>93</v>
       </c>
@@ -3546,7 +3547,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="68" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A68" s="2">
         <v>94</v>
       </c>
@@ -3584,7 +3585,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="69" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A69" s="2">
         <v>95</v>
       </c>
@@ -3622,7 +3623,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="70" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A70" s="2">
         <v>96</v>
       </c>
@@ -3660,7 +3661,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="71" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A71" s="2">
         <v>100</v>
       </c>
@@ -3698,7 +3699,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="72" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A72" s="2">
         <v>101</v>
       </c>
@@ -3736,7 +3737,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="73" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A73" s="2">
         <v>102</v>
       </c>
@@ -3774,7 +3775,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="74" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A74" s="2">
         <v>105</v>
       </c>
@@ -3812,7 +3813,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="75" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A75" s="2">
         <v>107</v>
       </c>
@@ -3850,7 +3851,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="76" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A76" s="2">
         <v>108</v>
       </c>
@@ -3888,7 +3889,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="77" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A77" s="2">
         <v>110</v>
       </c>
@@ -3926,7 +3927,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="78" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A78" s="2">
         <v>112</v>
       </c>
@@ -3964,7 +3965,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="79" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A79" s="2">
         <v>113</v>
       </c>
@@ -4002,7 +4003,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="80" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A80" s="2">
         <v>114</v>
       </c>
@@ -4040,7 +4041,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="81" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A81" s="2">
         <v>116</v>
       </c>
@@ -4078,7 +4079,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="82" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A82" s="2">
         <v>119</v>
       </c>
@@ -4116,7 +4117,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="83" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A83" s="2">
         <v>120</v>
       </c>
@@ -4154,7 +4155,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="84" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A84" s="2">
         <v>122</v>
       </c>
@@ -4192,7 +4193,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="85" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A85" s="2">
         <v>123</v>
       </c>
@@ -4230,7 +4231,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="86" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A86" s="2">
         <v>169</v>
       </c>
@@ -4268,7 +4269,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="87" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A87" s="2">
         <v>124</v>
       </c>
@@ -4306,7 +4307,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="88" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A88" s="2">
         <v>125</v>
       </c>
@@ -4344,7 +4345,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="89" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A89" s="2">
         <v>126</v>
       </c>
@@ -4382,7 +4383,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="90" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A90" s="2">
         <v>127</v>
       </c>
@@ -4420,7 +4421,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="91" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A91" s="2">
         <v>128</v>
       </c>
@@ -4458,7 +4459,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="92" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A92" s="2">
         <v>129</v>
       </c>
@@ -4496,7 +4497,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="93" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A93" s="2">
         <v>130</v>
       </c>
@@ -4534,7 +4535,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="94" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A94" s="2">
         <v>132</v>
       </c>
@@ -4572,7 +4573,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="95" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A95" s="2">
         <v>133</v>
       </c>
@@ -4610,7 +4611,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="96" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A96" s="2">
         <v>134</v>
       </c>
@@ -4648,7 +4649,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="97" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A97" s="2">
         <v>136</v>
       </c>
@@ -4686,7 +4687,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="98" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A98" s="2">
         <v>138</v>
       </c>
@@ -4724,7 +4725,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="99" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A99" s="2">
         <v>140</v>
       </c>
@@ -4762,7 +4763,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="100" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A100" s="2">
         <v>141</v>
       </c>
@@ -4800,7 +4801,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="101" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A101" s="2">
         <v>142</v>
       </c>
@@ -4838,7 +4839,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="102" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A102" s="2">
         <v>143</v>
       </c>
@@ -4876,7 +4877,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="103" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A103" s="2">
         <v>144</v>
       </c>
@@ -4914,7 +4915,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="104" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A104" s="2">
         <v>145</v>
       </c>
@@ -4952,7 +4953,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="105" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A105" s="2">
         <v>148</v>
       </c>
@@ -4990,7 +4991,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="106" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A106" s="2">
         <v>156</v>
       </c>
@@ -5026,7 +5027,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="107" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A107" s="2">
         <v>157</v>
       </c>
@@ -5062,7 +5063,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="108" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A108" s="2">
         <v>158</v>
       </c>
@@ -5100,7 +5101,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="109" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A109" s="2">
         <v>159</v>
       </c>
@@ -5136,7 +5137,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="110" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A110" s="2">
         <v>160</v>
       </c>
@@ -5172,7 +5173,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="111" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A111" s="2">
         <v>161</v>
       </c>
@@ -5208,7 +5209,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="112" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A112" s="2">
         <v>162</v>
       </c>
@@ -5244,7 +5245,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="113" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A113" s="2">
         <v>163</v>
       </c>
@@ -5280,7 +5281,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="114" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A114" s="2">
         <v>164</v>
       </c>
@@ -5316,7 +5317,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="115" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A115" s="2">
         <v>165</v>
       </c>
@@ -5354,7 +5355,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="116" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A116" s="2">
         <v>166</v>
       </c>
@@ -5390,7 +5391,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="117" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A117" s="2">
         <v>167</v>
       </c>
@@ -5426,7 +5427,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="118" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A118" s="2">
         <v>168</v>
       </c>
@@ -5464,7 +5465,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="119" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A119" s="2">
         <v>170</v>
       </c>
@@ -5502,7 +5503,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="120" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A120" s="2">
         <v>171</v>
       </c>
@@ -5540,7 +5541,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="121" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A121" s="2">
         <v>172</v>
       </c>
@@ -5578,7 +5579,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="122" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A122" s="2">
         <v>173</v>
       </c>
@@ -5616,7 +5617,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="123" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A123" s="2">
         <v>174</v>
       </c>
@@ -5654,7 +5655,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="124" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A124" s="2">
         <v>175</v>
       </c>
@@ -5692,7 +5693,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="125" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A125" s="2">
         <v>176</v>
       </c>
@@ -5730,7 +5731,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="126" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A126" s="2">
         <v>177</v>
       </c>
@@ -5768,7 +5769,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="127" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A127" s="2">
         <v>178</v>
       </c>
@@ -5806,7 +5807,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="128" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A128" s="2">
         <v>179</v>
       </c>
@@ -5844,7 +5845,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="129" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A129" s="2">
         <v>180</v>
       </c>
@@ -5882,7 +5883,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="130" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A130" s="2">
         <v>181</v>
       </c>
@@ -5920,7 +5921,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="131" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A131" s="2">
         <v>182</v>
       </c>
@@ -5958,7 +5959,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="132" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A132" s="2">
         <v>183</v>
       </c>
@@ -5996,7 +5997,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="133" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A133" s="2">
         <v>184</v>
       </c>
@@ -6032,7 +6033,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="134" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A134" s="2">
         <v>185</v>
       </c>
@@ -6068,7 +6069,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="135" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A135" s="2">
         <v>186</v>
       </c>
@@ -6104,7 +6105,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="136" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A136" s="2">
         <v>187</v>
       </c>
@@ -6140,7 +6141,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="137" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A137" s="2">
         <v>188</v>
       </c>
@@ -6178,7 +6179,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="138" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A138" s="2">
         <v>189</v>
       </c>
@@ -6216,7 +6217,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="139" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A139" s="2">
         <v>190</v>
       </c>
@@ -6254,7 +6255,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="140" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:12" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
       <c r="A140" s="2">
         <v>191</v>
       </c>
@@ -6292,7 +6293,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="141" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A141" s="2">
         <v>192</v>
       </c>
@@ -6331,6 +6332,13 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:L141" xr:uid="{B90B9044-5A84-4453-A4AB-9D3FAB58BBA5}">
+    <filterColumn colId="3">
+      <filters>
+        <filter val="COOPER STANDARD"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
 </file>

</xml_diff>